<commit_message>
update class use sbadmin2 css
</commit_message>
<xml_diff>
--- a/Documents/CandidateResponse.xlsx
+++ b/Documents/CandidateResponse.xlsx
@@ -8,15 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitLab\joboffer\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F1DA26D-548C-4B2B-B89C-4F9C26EBB347}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06A6D0AA-BA98-44F3-A763-08643446B591}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Responses" sheetId="1" r:id="rId1"/>
-    <sheet name="Samples" sheetId="2" r:id="rId2"/>
-    <sheet name="Sheet1" sheetId="3" r:id="rId3"/>
-    <sheet name="Sheet2" sheetId="4" r:id="rId4"/>
+    <sheet name="Sample" sheetId="5" r:id="rId2"/>
+    <sheet name="Mappings" sheetId="4" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="839" uniqueCount="329">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="508" uniqueCount="322">
   <si>
     <t>Id</t>
   </si>
@@ -566,87 +565,9 @@
     <t>cash for phone (worth 20k) with unli call, text, and data; ipad with unli data</t>
   </si>
   <si>
-    <t>anonymous</t>
-  </si>
-  <si>
-    <t>First Name Last Name 1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">14th and 15th month performance based-bonus </t>
-  </si>
-  <si>
-    <t>First Name Last Name 2</t>
-  </si>
-  <si>
-    <t>First Name Last Name 3</t>
-  </si>
-  <si>
-    <t>First Name Last Name 4</t>
-  </si>
-  <si>
-    <t>First Name Last Name 5</t>
-  </si>
-  <si>
-    <t>First Name Last Name 6</t>
-  </si>
-  <si>
-    <t>First Name Last Name 7</t>
-  </si>
-  <si>
-    <t>First Name Last Name 8</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Included in dental </t>
-  </si>
-  <si>
-    <t>First Name Last Name 9</t>
-  </si>
-  <si>
-    <t>First Name Last Name 10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Unilever </t>
-  </si>
-  <si>
-    <t>First Name Last Name 11</t>
-  </si>
-  <si>
-    <t>ECommerce Officer</t>
-  </si>
-  <si>
-    <t>WPP Media</t>
-  </si>
-  <si>
-    <t>Senior Associate - ECommerce Planning</t>
-  </si>
-  <si>
-    <t>800 php Phone Allowance</t>
-  </si>
-  <si>
-    <t>300000</t>
-  </si>
-  <si>
-    <t>200000</t>
-  </si>
-  <si>
-    <t>Up to 12,000 per year (x2 with dependent)</t>
-  </si>
-  <si>
-    <t>Medical reimbursements of PHP 15,000/year. Inclusive of PHP 12,500 Dental reimbursements.</t>
-  </si>
-  <si>
-    <t>15 days</t>
-  </si>
-  <si>
-    <t>Birthday leave - 1 day, emergency leave - 3 days</t>
-  </si>
-  <si>
     <t>₱500,000 coverage (company-paid)</t>
   </si>
   <si>
-    <t>Retirement Benefit • Marriage Bonus • Baby Bonus • Funeral Assistance</t>
-  </si>
-  <si>
     <t>alyssa.navarro@example.com</t>
   </si>
   <si>
@@ -710,9 +631,6 @@
     <t>Form field</t>
   </si>
   <si>
-    <t>Suggested column name</t>
-  </si>
-  <si>
     <t>ResponseStartedAt</t>
   </si>
   <si>
@@ -1023,6 +941,66 @@
   </si>
   <si>
     <t>rpaloma@example.com</t>
+  </si>
+  <si>
+    <t>DB Table column name</t>
+  </si>
+  <si>
+    <t>age</t>
+  </si>
+  <si>
+    <t>Components of Cash Compensation</t>
+  </si>
+  <si>
+    <t>C U R R E N T</t>
+  </si>
+  <si>
+    <t>OPTION 1</t>
+  </si>
+  <si>
+    <t>OPTION 2</t>
+  </si>
+  <si>
+    <t>OPTION 3</t>
+  </si>
+  <si>
+    <t>OPTION 4</t>
+  </si>
+  <si>
+    <t>Monthly</t>
+  </si>
+  <si>
+    <t>Annual</t>
+  </si>
+  <si>
+    <t>FIXED COMPONENT (Guaranteed Cash)</t>
+  </si>
+  <si>
+    <t>Monthly Basic Salary (MBS)</t>
+  </si>
+  <si>
+    <t>13th Month Pay (1.00 x MBS)</t>
+  </si>
+  <si>
+    <t>Other Guaranteed Bonus/es</t>
+  </si>
+  <si>
+    <t>Allowances</t>
+  </si>
+  <si>
+    <t>VARIABLE COMPONENT (Bonus/es)</t>
+  </si>
+  <si>
+    <t>Profit Share</t>
+  </si>
+  <si>
+    <t>Incentives/Commmission</t>
+  </si>
+  <si>
+    <t>Performance-Based Bonuses</t>
+  </si>
+  <si>
+    <t>GROSS COMPENSATION</t>
   </si>
 </sst>
 </file>
@@ -1060,15 +1038,21 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -1076,23 +1060,44 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1510,13 +1515,13 @@
         <v>46094.787835648203</v>
       </c>
       <c r="D2" t="s">
-        <v>203</v>
+        <v>177</v>
       </c>
       <c r="F2" t="s">
         <v>47</v>
       </c>
       <c r="G2" t="s">
-        <v>204</v>
+        <v>178</v>
       </c>
       <c r="H2">
         <v>46094</v>
@@ -1626,13 +1631,13 @@
         <v>46097.480868055602</v>
       </c>
       <c r="D3" t="s">
-        <v>205</v>
+        <v>179</v>
       </c>
       <c r="F3" t="s">
         <v>47</v>
       </c>
       <c r="G3" t="s">
-        <v>206</v>
+        <v>180</v>
       </c>
       <c r="H3">
         <v>46097</v>
@@ -1739,13 +1744,13 @@
         <v>46104.4124421296</v>
       </c>
       <c r="D4" t="s">
-        <v>207</v>
+        <v>181</v>
       </c>
       <c r="F4" t="s">
         <v>47</v>
       </c>
       <c r="G4" t="s">
-        <v>208</v>
+        <v>182</v>
       </c>
       <c r="H4">
         <v>46104</v>
@@ -1840,13 +1845,13 @@
         <v>46105.343738425901</v>
       </c>
       <c r="D5" t="s">
-        <v>209</v>
+        <v>183</v>
       </c>
       <c r="F5" t="s">
         <v>47</v>
       </c>
       <c r="G5" t="s">
-        <v>210</v>
+        <v>184</v>
       </c>
       <c r="H5">
         <v>46105</v>
@@ -1923,13 +1928,13 @@
         <v>46129.750752314802</v>
       </c>
       <c r="D6" t="s">
-        <v>211</v>
+        <v>185</v>
       </c>
       <c r="F6" t="s">
         <v>47</v>
       </c>
       <c r="G6" t="s">
-        <v>212</v>
+        <v>186</v>
       </c>
       <c r="H6">
         <v>46129</v>
@@ -2018,13 +2023,13 @@
         <v>46202.601712962998</v>
       </c>
       <c r="D7" t="s">
-        <v>213</v>
+        <v>187</v>
       </c>
       <c r="F7" t="s">
         <v>47</v>
       </c>
       <c r="G7" t="s">
-        <v>214</v>
+        <v>188</v>
       </c>
       <c r="H7">
         <v>46202</v>
@@ -2140,13 +2145,13 @@
         <v>46224.497453703698</v>
       </c>
       <c r="D8" t="s">
-        <v>215</v>
+        <v>189</v>
       </c>
       <c r="F8" t="s">
         <v>47</v>
       </c>
       <c r="G8" t="s">
-        <v>216</v>
+        <v>190</v>
       </c>
       <c r="H8">
         <v>46224</v>
@@ -2262,13 +2267,13 @@
         <v>46224.552905092598</v>
       </c>
       <c r="D9" t="s">
-        <v>217</v>
+        <v>191</v>
       </c>
       <c r="F9" t="s">
         <v>47</v>
       </c>
       <c r="G9" t="s">
-        <v>218</v>
+        <v>192</v>
       </c>
       <c r="H9">
         <v>46224</v>
@@ -2384,13 +2389,13 @@
         <v>46227.637407407397</v>
       </c>
       <c r="D10" t="s">
-        <v>219</v>
+        <v>193</v>
       </c>
       <c r="F10" t="s">
         <v>47</v>
       </c>
       <c r="G10" t="s">
-        <v>220</v>
+        <v>194</v>
       </c>
       <c r="H10">
         <v>46227</v>
@@ -2505,14 +2510,14 @@
       <c r="C11">
         <v>46227.731273148202</v>
       </c>
-      <c r="D11" s="4" t="s">
-        <v>221</v>
+      <c r="D11" s="3" t="s">
+        <v>195</v>
       </c>
       <c r="F11" t="s">
         <v>47</v>
       </c>
       <c r="G11" t="s">
-        <v>222</v>
+        <v>196</v>
       </c>
       <c r="H11">
         <v>46227</v>
@@ -2615,26 +2620,26 @@
       <c r="C12">
         <v>45689.615590277775</v>
       </c>
-      <c r="D12" s="4" t="s">
-        <v>325</v>
+      <c r="D12" s="3" t="s">
+        <v>298</v>
       </c>
       <c r="F12" t="s">
         <v>47</v>
       </c>
       <c r="G12" t="s">
-        <v>278</v>
+        <v>251</v>
       </c>
       <c r="H12">
         <v>45689</v>
       </c>
       <c r="I12" t="s">
-        <v>279</v>
+        <v>252</v>
       </c>
       <c r="K12">
         <v>44000</v>
       </c>
       <c r="L12" t="s">
-        <v>280</v>
+        <v>253</v>
       </c>
       <c r="M12" t="s">
         <v>82</v>
@@ -2643,19 +2648,19 @@
         <v>95</v>
       </c>
       <c r="O12" t="s">
-        <v>281</v>
+        <v>254</v>
       </c>
       <c r="P12" t="s">
         <v>109</v>
       </c>
       <c r="Q12" t="s">
-        <v>282</v>
+        <v>255</v>
       </c>
       <c r="R12">
         <v>22000</v>
       </c>
       <c r="S12" t="s">
-        <v>283</v>
+        <v>256</v>
       </c>
       <c r="T12" t="s">
         <v>100</v>
@@ -2664,7 +2669,7 @@
         <v>10000</v>
       </c>
       <c r="V12" t="s">
-        <v>284</v>
+        <v>257</v>
       </c>
       <c r="W12">
         <v>3000</v>
@@ -2676,7 +2681,7 @@
         <v>8000</v>
       </c>
       <c r="Z12" t="s">
-        <v>285</v>
+        <v>258</v>
       </c>
       <c r="AA12" t="s">
         <v>115</v>
@@ -2691,13 +2696,13 @@
         <v>36000</v>
       </c>
       <c r="AE12" t="s">
-        <v>286</v>
+        <v>259</v>
       </c>
       <c r="AF12">
         <v>0</v>
       </c>
       <c r="AG12" t="s">
-        <v>287</v>
+        <v>260</v>
       </c>
       <c r="AH12">
         <v>22000</v>
@@ -2706,28 +2711,28 @@
         <v>60</v>
       </c>
       <c r="AJ12" t="s">
-        <v>288</v>
+        <v>261</v>
       </c>
       <c r="AK12" t="s">
         <v>105</v>
       </c>
       <c r="AL12" t="s">
-        <v>289</v>
+        <v>262</v>
       </c>
       <c r="AM12" t="s">
-        <v>290</v>
+        <v>263</v>
       </c>
       <c r="AO12" t="s">
-        <v>291</v>
+        <v>264</v>
       </c>
       <c r="AP12" t="s">
-        <v>291</v>
+        <v>264</v>
       </c>
       <c r="AQ12" t="s">
-        <v>292</v>
+        <v>265</v>
       </c>
       <c r="AR12" t="s">
-        <v>201</v>
+        <v>176</v>
       </c>
     </row>
     <row r="13" spans="1:47">
@@ -2740,29 +2745,29 @@
       <c r="C13">
         <v>45689.631585648145</v>
       </c>
-      <c r="D13" s="4" t="s">
-        <v>326</v>
+      <c r="D13" s="3" t="s">
+        <v>299</v>
       </c>
       <c r="F13" t="s">
         <v>47</v>
       </c>
       <c r="G13" t="s">
-        <v>293</v>
+        <v>266</v>
       </c>
       <c r="H13">
         <v>45689</v>
       </c>
       <c r="I13" t="s">
-        <v>294</v>
+        <v>267</v>
       </c>
       <c r="J13" t="s">
-        <v>295</v>
+        <v>268</v>
       </c>
       <c r="K13">
         <v>40000</v>
       </c>
       <c r="L13" t="s">
-        <v>296</v>
+        <v>269</v>
       </c>
       <c r="M13" t="s">
         <v>82</v>
@@ -2771,19 +2776,19 @@
         <v>71</v>
       </c>
       <c r="O13" t="s">
-        <v>297</v>
+        <v>270</v>
       </c>
       <c r="P13" t="s">
         <v>127</v>
       </c>
       <c r="Q13" t="s">
-        <v>298</v>
+        <v>271</v>
       </c>
       <c r="R13">
         <v>40000</v>
       </c>
       <c r="S13" t="s">
-        <v>283</v>
+        <v>256</v>
       </c>
       <c r="T13" t="s">
         <v>100</v>
@@ -2792,7 +2797,7 @@
         <v>10000</v>
       </c>
       <c r="V13" t="s">
-        <v>284</v>
+        <v>257</v>
       </c>
       <c r="W13">
         <v>4000</v>
@@ -2804,13 +2809,13 @@
         <v>8000</v>
       </c>
       <c r="Z13" t="s">
-        <v>285</v>
+        <v>258</v>
       </c>
       <c r="AA13" t="s">
         <v>171</v>
       </c>
       <c r="AB13" t="s">
-        <v>299</v>
+        <v>272</v>
       </c>
       <c r="AC13">
         <v>7000</v>
@@ -2825,7 +2830,7 @@
         <v>0</v>
       </c>
       <c r="AG13" t="s">
-        <v>287</v>
+        <v>260</v>
       </c>
       <c r="AH13">
         <v>23000</v>
@@ -2834,7 +2839,7 @@
         <v>60</v>
       </c>
       <c r="AR13" t="s">
-        <v>300</v>
+        <v>273</v>
       </c>
     </row>
     <row r="14" spans="1:47">
@@ -2847,29 +2852,29 @@
       <c r="C14">
         <v>45689.677465277797</v>
       </c>
-      <c r="D14" s="4" t="s">
-        <v>327</v>
+      <c r="D14" s="3" t="s">
+        <v>300</v>
       </c>
       <c r="F14" t="s">
         <v>47</v>
       </c>
       <c r="G14" t="s">
-        <v>301</v>
+        <v>274</v>
       </c>
       <c r="H14">
         <v>45696</v>
       </c>
       <c r="I14" t="s">
-        <v>302</v>
+        <v>275</v>
       </c>
       <c r="J14" t="s">
-        <v>303</v>
+        <v>276</v>
       </c>
       <c r="K14">
         <v>50000</v>
       </c>
       <c r="L14" t="s">
-        <v>304</v>
+        <v>277</v>
       </c>
       <c r="M14" t="s">
         <v>82</v>
@@ -2878,13 +2883,13 @@
         <v>87</v>
       </c>
       <c r="O14" t="s">
-        <v>305</v>
+        <v>278</v>
       </c>
       <c r="P14" t="s">
-        <v>306</v>
+        <v>279</v>
       </c>
       <c r="Q14" t="s">
-        <v>307</v>
+        <v>280</v>
       </c>
       <c r="R14">
         <v>40000</v>
@@ -2899,7 +2904,7 @@
         <v>0</v>
       </c>
       <c r="V14" t="s">
-        <v>308</v>
+        <v>281</v>
       </c>
       <c r="W14">
         <v>2000</v>
@@ -2911,13 +2916,13 @@
         <v>8000</v>
       </c>
       <c r="Z14" t="s">
-        <v>285</v>
+        <v>258</v>
       </c>
       <c r="AA14">
         <v>1500</v>
       </c>
       <c r="AB14" t="s">
-        <v>299</v>
+        <v>272</v>
       </c>
       <c r="AC14">
         <v>12000</v>
@@ -2926,28 +2931,28 @@
         <v>60000</v>
       </c>
       <c r="AE14" t="s">
-        <v>286</v>
+        <v>259</v>
       </c>
       <c r="AF14">
         <v>80000</v>
       </c>
       <c r="AG14" t="s">
-        <v>287</v>
+        <v>260</v>
       </c>
       <c r="AH14">
         <v>20000</v>
       </c>
       <c r="AI14" t="s">
-        <v>309</v>
+        <v>282</v>
       </c>
       <c r="AJ14" t="s">
         <v>77</v>
       </c>
       <c r="AK14" t="s">
-        <v>310</v>
+        <v>283</v>
       </c>
       <c r="AL14" t="s">
-        <v>311</v>
+        <v>284</v>
       </c>
       <c r="AM14" t="s">
         <v>115</v>
@@ -2959,22 +2964,22 @@
         <v>106</v>
       </c>
       <c r="AP14" t="s">
-        <v>312</v>
+        <v>285</v>
       </c>
       <c r="AQ14" t="s">
-        <v>313</v>
+        <v>286</v>
       </c>
       <c r="AR14" t="s">
-        <v>314</v>
+        <v>287</v>
       </c>
       <c r="AS14" t="s">
         <v>55</v>
       </c>
       <c r="AT14" t="s">
-        <v>315</v>
+        <v>288</v>
       </c>
       <c r="AU14" t="s">
-        <v>316</v>
+        <v>289</v>
       </c>
     </row>
     <row r="15" spans="1:47">
@@ -2987,29 +2992,29 @@
       <c r="C15">
         <v>45690.5011689815</v>
       </c>
-      <c r="D15" s="4" t="s">
-        <v>328</v>
+      <c r="D15" s="3" t="s">
+        <v>301</v>
       </c>
       <c r="F15" t="s">
         <v>47</v>
       </c>
       <c r="G15" t="s">
-        <v>317</v>
+        <v>290</v>
       </c>
       <c r="H15">
         <v>45690</v>
       </c>
       <c r="I15" t="s">
-        <v>318</v>
+        <v>291</v>
       </c>
       <c r="J15" t="s">
-        <v>319</v>
+        <v>292</v>
       </c>
       <c r="K15">
         <v>40000</v>
       </c>
       <c r="L15" t="s">
-        <v>304</v>
+        <v>277</v>
       </c>
       <c r="M15" t="s">
         <v>82</v>
@@ -3018,19 +3023,19 @@
         <v>87</v>
       </c>
       <c r="O15" t="s">
-        <v>320</v>
+        <v>293</v>
       </c>
       <c r="P15" t="s">
         <v>127</v>
       </c>
       <c r="Q15" t="s">
-        <v>321</v>
+        <v>294</v>
       </c>
       <c r="R15">
         <v>48000</v>
       </c>
       <c r="S15" t="s">
-        <v>283</v>
+        <v>256</v>
       </c>
       <c r="T15" t="s">
         <v>100</v>
@@ -3039,25 +3044,25 @@
         <v>5000</v>
       </c>
       <c r="V15" t="s">
-        <v>308</v>
+        <v>281</v>
       </c>
       <c r="W15">
         <v>2000</v>
       </c>
       <c r="X15" t="s">
-        <v>322</v>
+        <v>295</v>
       </c>
       <c r="Y15">
         <v>8000</v>
       </c>
       <c r="Z15" t="s">
-        <v>323</v>
+        <v>296</v>
       </c>
       <c r="AA15">
         <v>0</v>
       </c>
       <c r="AB15" t="s">
-        <v>323</v>
+        <v>296</v>
       </c>
       <c r="AC15">
         <v>0</v>
@@ -3066,13 +3071,13 @@
         <v>40000</v>
       </c>
       <c r="AE15" t="s">
-        <v>323</v>
+        <v>296</v>
       </c>
       <c r="AF15">
         <v>0</v>
       </c>
       <c r="AG15" t="s">
-        <v>324</v>
+        <v>297</v>
       </c>
       <c r="AH15">
         <v>0</v>
@@ -3091,1367 +3096,354 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:AU12"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{736AB341-0D96-4F08-9924-0422DE3D22D2}">
+  <dimension ref="B3:M15"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
+  <cols>
+    <col min="2" max="2" width="33.08984375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.90625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="6.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.6328125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="6.81640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="8.6328125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="7.81640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="8.6328125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="7.81640625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8.6328125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="7.81640625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:47">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" t="s">
-        <v>8</v>
-      </c>
-      <c r="J1" t="s">
-        <v>9</v>
-      </c>
-      <c r="K1" t="s">
-        <v>10</v>
-      </c>
-      <c r="L1" t="s">
-        <v>11</v>
-      </c>
-      <c r="M1" t="s">
-        <v>12</v>
-      </c>
-      <c r="N1" t="s">
-        <v>13</v>
-      </c>
-      <c r="O1" t="s">
-        <v>14</v>
-      </c>
-      <c r="P1" t="s">
-        <v>15</v>
-      </c>
-      <c r="Q1" t="s">
-        <v>16</v>
-      </c>
-      <c r="R1" t="s">
-        <v>17</v>
-      </c>
-      <c r="S1" t="s">
-        <v>18</v>
-      </c>
-      <c r="T1" t="s">
-        <v>19</v>
-      </c>
-      <c r="U1" t="s">
-        <v>20</v>
-      </c>
-      <c r="V1" t="s">
-        <v>21</v>
-      </c>
-      <c r="W1" t="s">
-        <v>22</v>
-      </c>
-      <c r="X1" t="s">
-        <v>23</v>
-      </c>
-      <c r="Y1" t="s">
-        <v>24</v>
-      </c>
-      <c r="Z1" t="s">
-        <v>25</v>
-      </c>
-      <c r="AA1" t="s">
-        <v>26</v>
-      </c>
-      <c r="AB1" t="s">
-        <v>27</v>
-      </c>
-      <c r="AC1" t="s">
-        <v>28</v>
-      </c>
-      <c r="AD1" t="s">
-        <v>29</v>
-      </c>
-      <c r="AE1" t="s">
-        <v>30</v>
-      </c>
-      <c r="AF1" t="s">
-        <v>31</v>
-      </c>
-      <c r="AG1" t="s">
-        <v>32</v>
-      </c>
-      <c r="AH1" t="s">
-        <v>33</v>
-      </c>
-      <c r="AI1" t="s">
-        <v>34</v>
-      </c>
-      <c r="AJ1" t="s">
-        <v>35</v>
-      </c>
-      <c r="AK1" t="s">
-        <v>36</v>
-      </c>
-      <c r="AL1" t="s">
-        <v>37</v>
-      </c>
-      <c r="AM1" t="s">
-        <v>38</v>
-      </c>
-      <c r="AN1" t="s">
-        <v>39</v>
-      </c>
-      <c r="AO1" t="s">
-        <v>40</v>
-      </c>
-      <c r="AP1" t="s">
-        <v>41</v>
-      </c>
-      <c r="AQ1" t="s">
-        <v>42</v>
-      </c>
-      <c r="AR1" t="s">
-        <v>43</v>
-      </c>
-      <c r="AS1" t="s">
-        <v>44</v>
-      </c>
-      <c r="AT1" t="s">
-        <v>45</v>
-      </c>
-      <c r="AU1" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="2" spans="1:47">
-      <c r="A2">
-        <v>34</v>
-      </c>
-      <c r="B2">
-        <v>46094.707060185203</v>
-      </c>
-      <c r="C2">
-        <v>46094.787835648203</v>
-      </c>
-      <c r="D2" t="s">
-        <v>176</v>
-      </c>
-      <c r="F2" t="s">
-        <v>47</v>
-      </c>
-      <c r="G2" t="s">
-        <v>177</v>
-      </c>
-      <c r="H2">
-        <v>46094</v>
-      </c>
-      <c r="I2" t="s">
-        <v>48</v>
-      </c>
-      <c r="K2">
-        <v>120000</v>
-      </c>
-      <c r="M2" t="s">
-        <v>49</v>
-      </c>
-      <c r="N2" t="s">
-        <v>50</v>
-      </c>
-      <c r="O2" t="s">
-        <v>51</v>
-      </c>
-      <c r="P2" t="s">
-        <v>52</v>
-      </c>
-      <c r="Q2" t="s">
-        <v>53</v>
-      </c>
-      <c r="R2">
-        <v>83530</v>
-      </c>
-      <c r="S2" t="s">
-        <v>54</v>
-      </c>
-      <c r="T2" t="s">
-        <v>55</v>
-      </c>
-      <c r="U2">
-        <v>83530</v>
-      </c>
-      <c r="V2" t="s">
-        <v>56</v>
-      </c>
-      <c r="W2">
-        <v>5640</v>
-      </c>
-      <c r="X2" t="s">
-        <v>57</v>
-      </c>
-      <c r="Y2">
-        <v>11000</v>
-      </c>
-      <c r="AD2">
-        <v>0</v>
-      </c>
-      <c r="AE2" t="s">
-        <v>58</v>
-      </c>
-      <c r="AF2">
-        <v>144000</v>
-      </c>
-      <c r="AG2" t="s">
-        <v>178</v>
-      </c>
-      <c r="AH2">
-        <v>167060</v>
-      </c>
-      <c r="AI2" t="s">
-        <v>60</v>
-      </c>
-      <c r="AJ2" t="s">
-        <v>61</v>
-      </c>
-      <c r="AK2" t="s">
-        <v>62</v>
-      </c>
-      <c r="AL2" t="s">
-        <v>63</v>
-      </c>
-      <c r="AM2" t="s">
-        <v>64</v>
-      </c>
-      <c r="AN2" t="s">
-        <v>55</v>
-      </c>
-      <c r="AO2" t="s">
-        <v>65</v>
-      </c>
-      <c r="AP2" t="s">
-        <v>66</v>
-      </c>
-      <c r="AQ2" t="s">
-        <v>55</v>
-      </c>
-      <c r="AR2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AS2" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="3" spans="1:47">
-      <c r="A3">
-        <v>35</v>
-      </c>
-      <c r="B3">
-        <v>46097.459386574097</v>
-      </c>
-      <c r="C3">
-        <v>46097.480868055602</v>
-      </c>
-      <c r="D3" t="s">
-        <v>176</v>
+    <row r="3" spans="2:13">
+      <c r="B3" t="s">
+        <v>304</v>
+      </c>
+      <c r="C3" t="s">
+        <v>305</v>
       </c>
       <c r="F3" t="s">
-        <v>47</v>
-      </c>
-      <c r="G3" t="s">
-        <v>179</v>
-      </c>
-      <c r="H3">
-        <v>46097</v>
-      </c>
-      <c r="I3" t="s">
-        <v>69</v>
-      </c>
-      <c r="K3">
+        <v>306</v>
+      </c>
+      <c r="H3" t="s">
+        <v>307</v>
+      </c>
+      <c r="J3" t="s">
+        <v>308</v>
+      </c>
+      <c r="L3" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="4" spans="2:13">
+      <c r="C4" t="s">
+        <v>310</v>
+      </c>
+      <c r="D4" t="s">
+        <v>311</v>
+      </c>
+      <c r="F4" t="s">
+        <v>310</v>
+      </c>
+      <c r="G4" t="s">
+        <v>311</v>
+      </c>
+      <c r="H4" t="s">
+        <v>310</v>
+      </c>
+      <c r="I4" t="s">
+        <v>311</v>
+      </c>
+      <c r="J4" t="s">
+        <v>310</v>
+      </c>
+      <c r="K4" t="s">
+        <v>311</v>
+      </c>
+      <c r="L4" t="s">
+        <v>310</v>
+      </c>
+      <c r="M4" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="5" spans="2:13">
+      <c r="B5" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="6" spans="2:13">
+      <c r="B6" t="s">
+        <v>313</v>
+      </c>
+      <c r="C6">
+        <v>22000</v>
+      </c>
+      <c r="D6">
+        <v>264000</v>
+      </c>
+      <c r="F6">
         <v>55000</v>
       </c>
-      <c r="M3" t="s">
-        <v>70</v>
-      </c>
-      <c r="N3" t="s">
-        <v>71</v>
-      </c>
-      <c r="O3" t="s">
-        <v>72</v>
-      </c>
-      <c r="P3" t="s">
-        <v>73</v>
-      </c>
-      <c r="Q3" t="s">
-        <v>74</v>
-      </c>
-      <c r="R3">
-        <v>45500</v>
-      </c>
-      <c r="S3" t="s">
-        <v>54</v>
-      </c>
-      <c r="T3" t="s">
-        <v>55</v>
-      </c>
-      <c r="U3">
-        <v>0</v>
-      </c>
-      <c r="V3" t="s">
-        <v>75</v>
-      </c>
-      <c r="W3">
-        <v>2500</v>
-      </c>
-      <c r="X3" t="s">
-        <v>55</v>
-      </c>
-      <c r="Y3">
-        <v>0</v>
-      </c>
-      <c r="AD3">
-        <v>0</v>
-      </c>
-      <c r="AE3" t="s">
-        <v>55</v>
-      </c>
-      <c r="AF3">
-        <v>0</v>
-      </c>
-      <c r="AG3" t="s">
-        <v>76</v>
-      </c>
-      <c r="AH3">
-        <v>24735.56</v>
-      </c>
-      <c r="AI3" t="s">
-        <v>77</v>
-      </c>
-      <c r="AJ3" t="s">
-        <v>55</v>
-      </c>
-      <c r="AK3" t="s">
-        <v>78</v>
-      </c>
-      <c r="AL3" t="s">
-        <v>61</v>
-      </c>
-      <c r="AM3" t="s">
-        <v>61</v>
-      </c>
-      <c r="AN3" t="s">
-        <v>61</v>
-      </c>
-      <c r="AO3" t="s">
-        <v>79</v>
-      </c>
-      <c r="AP3" t="s">
-        <v>80</v>
-      </c>
-      <c r="AQ3" t="s">
-        <v>55</v>
-      </c>
-      <c r="AR3" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="4" spans="1:47">
-      <c r="A4">
-        <v>36</v>
-      </c>
-      <c r="B4">
-        <v>46104.409814814797</v>
-      </c>
-      <c r="C4">
-        <v>46104.4124421296</v>
-      </c>
-      <c r="D4" t="s">
-        <v>176</v>
-      </c>
-      <c r="F4" t="s">
-        <v>47</v>
-      </c>
-      <c r="G4" t="s">
-        <v>180</v>
-      </c>
-      <c r="H4">
-        <v>46104</v>
-      </c>
-      <c r="I4" t="s">
-        <v>81</v>
-      </c>
-      <c r="K4">
-        <v>180000</v>
-      </c>
-      <c r="M4" t="s">
-        <v>82</v>
-      </c>
-      <c r="N4" t="s">
-        <v>50</v>
-      </c>
-      <c r="O4" t="s">
-        <v>83</v>
-      </c>
-      <c r="P4" t="s">
-        <v>52</v>
-      </c>
-      <c r="Q4" t="s">
-        <v>84</v>
-      </c>
-      <c r="R4">
-        <v>90000</v>
-      </c>
-      <c r="S4" t="s">
-        <v>54</v>
-      </c>
-      <c r="V4">
-        <v>0</v>
-      </c>
-      <c r="W4">
-        <v>0</v>
-      </c>
-      <c r="X4">
-        <v>0</v>
-      </c>
-      <c r="Y4">
-        <v>0</v>
-      </c>
-      <c r="AD4">
-        <v>0</v>
-      </c>
-      <c r="AE4" t="s">
-        <v>85</v>
-      </c>
-      <c r="AH4">
-        <v>0</v>
-      </c>
-      <c r="AI4" t="s">
-        <v>61</v>
-      </c>
-      <c r="AJ4" t="s">
-        <v>61</v>
-      </c>
-      <c r="AK4" t="s">
-        <v>61</v>
-      </c>
-      <c r="AL4" t="s">
-        <v>61</v>
-      </c>
-      <c r="AM4" t="s">
-        <v>61</v>
-      </c>
-      <c r="AN4" t="s">
-        <v>61</v>
-      </c>
-      <c r="AO4" t="s">
-        <v>61</v>
-      </c>
-      <c r="AP4" t="s">
-        <v>61</v>
-      </c>
-      <c r="AQ4" t="s">
-        <v>61</v>
-      </c>
-      <c r="AR4" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="5" spans="1:47">
-      <c r="A5">
-        <v>37</v>
-      </c>
-      <c r="B5">
-        <v>46105.328229166698</v>
-      </c>
-      <c r="C5">
-        <v>46105.343738425901</v>
-      </c>
-      <c r="D5" t="s">
-        <v>176</v>
-      </c>
-      <c r="F5" t="s">
-        <v>47</v>
-      </c>
-      <c r="G5" t="s">
-        <v>181</v>
-      </c>
-      <c r="H5">
-        <v>46105</v>
-      </c>
-      <c r="I5" t="s">
-        <v>86</v>
-      </c>
-      <c r="K5">
-        <v>45000</v>
-      </c>
-      <c r="M5" t="s">
-        <v>49</v>
-      </c>
-      <c r="N5" t="s">
-        <v>87</v>
-      </c>
-      <c r="O5" t="s">
-        <v>88</v>
-      </c>
-      <c r="P5" t="s">
-        <v>89</v>
-      </c>
-      <c r="Q5" t="s">
-        <v>90</v>
-      </c>
-      <c r="R5">
-        <v>45000</v>
-      </c>
-      <c r="S5" t="s">
-        <v>91</v>
-      </c>
-      <c r="T5" t="s">
-        <v>92</v>
-      </c>
-      <c r="U5">
-        <v>30000</v>
-      </c>
-      <c r="V5" t="s">
-        <v>55</v>
-      </c>
-      <c r="W5">
-        <v>0</v>
-      </c>
-      <c r="X5" t="s">
-        <v>93</v>
-      </c>
-      <c r="Y5">
-        <v>0</v>
-      </c>
-      <c r="AD5">
-        <v>0</v>
-      </c>
-      <c r="AE5">
-        <v>180000</v>
-      </c>
-      <c r="AF5">
-        <v>180000</v>
-      </c>
-      <c r="AG5" t="s">
-        <v>93</v>
-      </c>
-      <c r="AH5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:47">
-      <c r="A6">
-        <v>38</v>
-      </c>
-      <c r="B6">
-        <v>46129.722800925898</v>
-      </c>
-      <c r="C6">
-        <v>46129.750752314802</v>
-      </c>
-      <c r="D6" t="s">
-        <v>176</v>
-      </c>
-      <c r="F6" t="s">
-        <v>47</v>
-      </c>
-      <c r="G6" t="s">
-        <v>182</v>
+      <c r="G6">
+        <v>660000</v>
       </c>
       <c r="H6">
-        <v>46129</v>
-      </c>
-      <c r="I6" t="s">
-        <v>94</v>
+        <v>65000</v>
+      </c>
+      <c r="I6">
+        <v>780000</v>
+      </c>
+      <c r="J6">
+        <v>77000</v>
       </c>
       <c r="K6">
-        <v>35000</v>
-      </c>
-      <c r="M6" t="s">
-        <v>82</v>
-      </c>
-      <c r="N6" t="s">
-        <v>95</v>
-      </c>
-      <c r="O6" t="s">
-        <v>96</v>
-      </c>
-      <c r="P6" t="s">
-        <v>97</v>
-      </c>
-      <c r="Q6" t="s">
-        <v>98</v>
-      </c>
-      <c r="R6">
+        <v>924000</v>
+      </c>
+      <c r="L6">
+        <v>80000</v>
+      </c>
+      <c r="M6">
+        <v>960000</v>
+      </c>
+    </row>
+    <row r="7" spans="2:13">
+      <c r="B7" t="s">
+        <v>314</v>
+      </c>
+      <c r="C7">
+        <v>0</v>
+      </c>
+      <c r="D7">
+        <v>22000</v>
+      </c>
+      <c r="F7">
+        <v>0</v>
+      </c>
+      <c r="G7">
+        <v>55000</v>
+      </c>
+      <c r="H7">
+        <v>0</v>
+      </c>
+      <c r="I7">
+        <v>65000</v>
+      </c>
+      <c r="J7">
+        <v>0</v>
+      </c>
+      <c r="K7">
+        <v>77000</v>
+      </c>
+      <c r="L7">
+        <v>0</v>
+      </c>
+      <c r="M7">
+        <v>80000</v>
+      </c>
+    </row>
+    <row r="8" spans="2:13">
+      <c r="B8" t="s">
+        <v>315</v>
+      </c>
+      <c r="C8">
+        <v>0</v>
+      </c>
+      <c r="D8">
+        <v>10000</v>
+      </c>
+      <c r="F8">
+        <v>0</v>
+      </c>
+      <c r="G8">
+        <v>110000</v>
+      </c>
+      <c r="H8">
+        <v>0</v>
+      </c>
+      <c r="I8">
+        <v>130000</v>
+      </c>
+      <c r="J8">
+        <v>0</v>
+      </c>
+      <c r="K8">
+        <v>154000</v>
+      </c>
+      <c r="L8">
+        <v>0</v>
+      </c>
+      <c r="M8">
+        <v>160000</v>
+      </c>
+    </row>
+    <row r="9" spans="2:13">
+      <c r="B9" t="s">
+        <v>316</v>
+      </c>
+      <c r="C9">
+        <v>0</v>
+      </c>
+      <c r="D9">
         <v>25000</v>
       </c>
-      <c r="S6" t="s">
-        <v>99</v>
-      </c>
-      <c r="T6" t="s">
-        <v>100</v>
-      </c>
-      <c r="U6">
-        <v>10000</v>
-      </c>
-      <c r="V6" t="s">
-        <v>101</v>
-      </c>
-      <c r="W6">
-        <v>3600</v>
-      </c>
-      <c r="X6" t="s">
-        <v>102</v>
-      </c>
-      <c r="Y6">
-        <v>2500</v>
-      </c>
-      <c r="AD6">
-        <v>0</v>
-      </c>
-      <c r="AE6" t="s">
-        <v>103</v>
-      </c>
-      <c r="AF6">
-        <v>0</v>
-      </c>
-      <c r="AG6" t="s">
-        <v>103</v>
-      </c>
-      <c r="AH6">
-        <v>0</v>
-      </c>
-      <c r="AI6" t="s">
-        <v>104</v>
-      </c>
-      <c r="AK6" t="s">
-        <v>105</v>
-      </c>
-      <c r="AO6" t="s">
-        <v>106</v>
-      </c>
-      <c r="AP6" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="7" spans="1:47">
-      <c r="A7">
-        <v>39</v>
-      </c>
-      <c r="B7">
-        <v>46202.589166666701</v>
-      </c>
-      <c r="C7">
-        <v>46202.601712962998</v>
-      </c>
-      <c r="D7" t="s">
-        <v>176</v>
-      </c>
-      <c r="F7" t="s">
-        <v>47</v>
-      </c>
-      <c r="G7" t="s">
-        <v>183</v>
-      </c>
-      <c r="H7">
-        <v>46202</v>
-      </c>
-      <c r="I7" t="s">
-        <v>107</v>
-      </c>
-      <c r="K7">
+      <c r="F9">
+        <v>4062.5</v>
+      </c>
+      <c r="G9">
+        <v>48750</v>
+      </c>
+      <c r="H9">
+        <v>4062.5</v>
+      </c>
+      <c r="I9">
+        <v>48750</v>
+      </c>
+      <c r="J9">
+        <v>4062.5</v>
+      </c>
+      <c r="K9">
+        <v>48750</v>
+      </c>
+      <c r="L9">
+        <v>4062.5</v>
+      </c>
+      <c r="M9">
+        <v>48750</v>
+      </c>
+    </row>
+    <row r="11" spans="2:13">
+      <c r="B11" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="12" spans="2:13">
+      <c r="B12" t="s">
+        <v>318</v>
+      </c>
+      <c r="C12">
+        <v>0</v>
+      </c>
+      <c r="D12">
+        <v>36000</v>
+      </c>
+      <c r="F12">
+        <v>0</v>
+      </c>
+      <c r="G12">
+        <v>55000</v>
+      </c>
+      <c r="H12">
+        <v>0</v>
+      </c>
+      <c r="I12">
         <v>65000</v>
       </c>
-      <c r="M7" t="s">
-        <v>82</v>
-      </c>
-      <c r="N7" t="s">
-        <v>50</v>
-      </c>
-      <c r="O7" t="s">
-        <v>108</v>
-      </c>
-      <c r="P7" t="s">
-        <v>109</v>
-      </c>
-      <c r="Q7" t="s">
-        <v>110</v>
-      </c>
-      <c r="R7">
-        <v>60000</v>
-      </c>
-      <c r="S7" t="s">
-        <v>91</v>
-      </c>
-      <c r="T7" t="s">
-        <v>111</v>
-      </c>
-      <c r="U7">
-        <v>60000</v>
-      </c>
-      <c r="V7" t="s">
-        <v>112</v>
-      </c>
-      <c r="W7">
-        <v>25000</v>
-      </c>
-      <c r="X7" t="s">
-        <v>55</v>
-      </c>
-      <c r="Y7">
-        <v>0</v>
-      </c>
-      <c r="AD7">
-        <v>0</v>
-      </c>
-      <c r="AE7" t="s">
-        <v>113</v>
-      </c>
-      <c r="AF7">
-        <v>10000</v>
-      </c>
-      <c r="AG7" t="s">
-        <v>55</v>
-      </c>
-      <c r="AH7">
-        <v>0</v>
-      </c>
-      <c r="AI7" t="s">
-        <v>114</v>
-      </c>
-      <c r="AJ7" t="s">
-        <v>114</v>
-      </c>
-      <c r="AK7" t="s">
-        <v>115</v>
-      </c>
-      <c r="AL7" t="s">
-        <v>116</v>
-      </c>
-      <c r="AM7" t="s">
-        <v>55</v>
-      </c>
-      <c r="AN7" t="s">
-        <v>55</v>
-      </c>
-      <c r="AO7" t="s">
-        <v>117</v>
-      </c>
-      <c r="AP7" t="s">
-        <v>118</v>
-      </c>
-      <c r="AQ7" t="s">
-        <v>119</v>
-      </c>
-      <c r="AR7" t="s">
-        <v>120</v>
-      </c>
-      <c r="AS7" t="s">
-        <v>121</v>
-      </c>
-      <c r="AT7" t="s">
-        <v>122</v>
-      </c>
-      <c r="AU7" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="8" spans="1:47">
-      <c r="A8">
-        <v>40</v>
-      </c>
-      <c r="B8">
-        <v>46224.478032407402</v>
-      </c>
-      <c r="C8">
-        <v>46224.497453703698</v>
-      </c>
-      <c r="D8" t="s">
-        <v>176</v>
-      </c>
-      <c r="F8" t="s">
-        <v>47</v>
-      </c>
-      <c r="G8" t="s">
-        <v>184</v>
-      </c>
-      <c r="H8">
-        <v>46224</v>
-      </c>
-      <c r="I8" t="s">
-        <v>124</v>
-      </c>
-      <c r="K8">
-        <v>75000</v>
-      </c>
-      <c r="M8" t="s">
-        <v>82</v>
-      </c>
-      <c r="N8" t="s">
-        <v>125</v>
-      </c>
-      <c r="O8" t="s">
-        <v>126</v>
-      </c>
-      <c r="P8" t="s">
-        <v>127</v>
-      </c>
-      <c r="Q8" t="s">
-        <v>128</v>
-      </c>
-      <c r="R8">
-        <v>56450</v>
-      </c>
-      <c r="S8" t="s">
-        <v>54</v>
-      </c>
-      <c r="T8" t="s">
-        <v>129</v>
-      </c>
-      <c r="U8">
-        <v>60000</v>
-      </c>
-      <c r="V8" t="s">
-        <v>130</v>
-      </c>
-      <c r="W8">
-        <v>3550</v>
-      </c>
-      <c r="X8" t="s">
-        <v>55</v>
-      </c>
-      <c r="Y8">
-        <v>0</v>
-      </c>
-      <c r="AD8">
-        <v>0</v>
-      </c>
-      <c r="AE8" t="s">
-        <v>55</v>
-      </c>
-      <c r="AF8">
-        <v>0</v>
-      </c>
-      <c r="AG8">
-        <v>0</v>
-      </c>
-      <c r="AH8">
-        <v>0</v>
-      </c>
-      <c r="AI8" t="s">
-        <v>131</v>
-      </c>
-      <c r="AJ8" t="s">
-        <v>61</v>
-      </c>
-      <c r="AK8" t="s">
-        <v>105</v>
-      </c>
-      <c r="AL8" t="s">
-        <v>132</v>
-      </c>
-      <c r="AM8" t="s">
-        <v>132</v>
-      </c>
-      <c r="AN8" t="s">
-        <v>61</v>
-      </c>
-      <c r="AO8" t="s">
-        <v>133</v>
-      </c>
-      <c r="AP8" t="s">
-        <v>134</v>
-      </c>
-      <c r="AQ8" t="s">
-        <v>61</v>
-      </c>
-      <c r="AR8" t="s">
-        <v>61</v>
-      </c>
-      <c r="AS8" t="s">
-        <v>135</v>
-      </c>
-      <c r="AT8" t="s">
-        <v>61</v>
-      </c>
-      <c r="AU8" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="9" spans="1:47">
-      <c r="A9">
-        <v>41</v>
-      </c>
-      <c r="B9">
-        <v>46224.533090277801</v>
-      </c>
-      <c r="C9">
-        <v>46224.552905092598</v>
-      </c>
-      <c r="D9" t="s">
-        <v>176</v>
-      </c>
-      <c r="F9" t="s">
-        <v>47</v>
-      </c>
-      <c r="G9" t="s">
-        <v>185</v>
-      </c>
-      <c r="H9">
-        <v>46224</v>
-      </c>
-      <c r="I9" t="s">
-        <v>136</v>
-      </c>
-      <c r="K9">
-        <v>60000</v>
-      </c>
-      <c r="M9" t="s">
-        <v>49</v>
-      </c>
-      <c r="N9" t="s">
-        <v>125</v>
-      </c>
-      <c r="O9" t="s">
-        <v>137</v>
-      </c>
-      <c r="P9" t="s">
-        <v>138</v>
-      </c>
-      <c r="Q9" t="s">
-        <v>139</v>
-      </c>
-      <c r="R9">
-        <v>25000</v>
-      </c>
-      <c r="S9" t="s">
-        <v>54</v>
-      </c>
-      <c r="T9" t="s">
-        <v>55</v>
-      </c>
-      <c r="U9">
-        <v>0</v>
-      </c>
-      <c r="V9" t="s">
-        <v>140</v>
-      </c>
-      <c r="W9">
-        <v>1250</v>
-      </c>
-      <c r="X9" t="s">
-        <v>141</v>
-      </c>
-      <c r="Y9">
-        <v>1500</v>
-      </c>
-      <c r="AD9">
-        <v>25000</v>
-      </c>
-      <c r="AE9" t="s">
-        <v>55</v>
-      </c>
-      <c r="AF9">
-        <v>0</v>
-      </c>
-      <c r="AG9" t="s">
-        <v>55</v>
-      </c>
-      <c r="AH9">
-        <v>0</v>
-      </c>
-      <c r="AI9" t="s">
-        <v>142</v>
-      </c>
-      <c r="AJ9" t="s">
-        <v>142</v>
-      </c>
-      <c r="AK9" t="s">
-        <v>143</v>
-      </c>
-      <c r="AL9" t="s">
-        <v>186</v>
-      </c>
-      <c r="AM9" t="s">
-        <v>144</v>
-      </c>
-      <c r="AN9" t="s">
-        <v>55</v>
-      </c>
-      <c r="AO9" t="s">
-        <v>145</v>
-      </c>
-      <c r="AP9" t="s">
-        <v>146</v>
-      </c>
-      <c r="AQ9" t="s">
-        <v>55</v>
-      </c>
-      <c r="AR9" t="s">
-        <v>55</v>
-      </c>
-      <c r="AS9" t="s">
-        <v>55</v>
-      </c>
-      <c r="AT9" t="s">
-        <v>55</v>
-      </c>
-      <c r="AU9" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="10" spans="1:47">
-      <c r="A10">
-        <v>42</v>
-      </c>
-      <c r="B10">
-        <v>46227.628240740698</v>
-      </c>
-      <c r="C10">
-        <v>46227.637407407397</v>
-      </c>
-      <c r="D10" t="s">
-        <v>176</v>
-      </c>
-      <c r="F10" t="s">
-        <v>47</v>
-      </c>
-      <c r="G10" t="s">
-        <v>187</v>
-      </c>
-      <c r="H10">
-        <v>46227</v>
-      </c>
-      <c r="I10" t="s">
-        <v>147</v>
-      </c>
-      <c r="K10">
-        <v>140000</v>
-      </c>
-      <c r="M10" t="s">
-        <v>49</v>
-      </c>
-      <c r="N10" t="s">
-        <v>87</v>
-      </c>
-      <c r="O10" t="s">
-        <v>148</v>
-      </c>
-      <c r="P10" t="s">
-        <v>89</v>
-      </c>
-      <c r="Q10" t="s">
-        <v>149</v>
-      </c>
-      <c r="R10">
-        <v>85079.63</v>
-      </c>
-      <c r="S10" t="s">
-        <v>54</v>
-      </c>
-      <c r="T10" t="s">
-        <v>55</v>
-      </c>
-      <c r="U10">
-        <v>0</v>
-      </c>
-      <c r="V10" t="s">
-        <v>150</v>
-      </c>
-      <c r="W10">
-        <v>6000</v>
-      </c>
-      <c r="X10" t="s">
-        <v>151</v>
-      </c>
-      <c r="Y10">
-        <v>8000</v>
-      </c>
-      <c r="AD10">
-        <v>0</v>
-      </c>
-      <c r="AE10" t="s">
-        <v>152</v>
-      </c>
-      <c r="AF10">
-        <v>320000</v>
-      </c>
-      <c r="AG10" t="s">
-        <v>55</v>
-      </c>
-      <c r="AH10">
-        <v>0</v>
-      </c>
-      <c r="AI10" t="s">
-        <v>153</v>
-      </c>
-      <c r="AJ10" t="s">
-        <v>154</v>
-      </c>
-      <c r="AK10" t="s">
-        <v>105</v>
-      </c>
-      <c r="AL10" t="s">
-        <v>55</v>
-      </c>
-      <c r="AM10" t="s">
-        <v>155</v>
-      </c>
-      <c r="AN10" t="s">
-        <v>55</v>
-      </c>
-      <c r="AO10" t="s">
-        <v>156</v>
-      </c>
-      <c r="AP10" t="s">
-        <v>157</v>
-      </c>
-      <c r="AQ10" t="s">
-        <v>55</v>
-      </c>
-      <c r="AR10" t="s">
-        <v>55</v>
-      </c>
-      <c r="AS10" t="s">
-        <v>158</v>
-      </c>
-      <c r="AT10" t="s">
-        <v>159</v>
-      </c>
-      <c r="AU10" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="11" spans="1:47">
-      <c r="A11">
-        <v>43</v>
-      </c>
-      <c r="B11">
-        <v>46227.686967592599</v>
-      </c>
-      <c r="C11">
-        <v>46227.731273148202</v>
-      </c>
-      <c r="D11" t="s">
-        <v>176</v>
-      </c>
-      <c r="F11" t="s">
-        <v>47</v>
-      </c>
-      <c r="G11" t="s">
-        <v>188</v>
-      </c>
-      <c r="H11">
-        <v>46227</v>
-      </c>
-      <c r="I11" t="s">
-        <v>161</v>
-      </c>
-      <c r="K11">
-        <v>90000</v>
-      </c>
-      <c r="M11" t="s">
-        <v>82</v>
-      </c>
-      <c r="N11" t="s">
-        <v>87</v>
-      </c>
-      <c r="O11" t="s">
-        <v>189</v>
-      </c>
-      <c r="P11" t="s">
-        <v>89</v>
-      </c>
-      <c r="Q11" t="s">
-        <v>163</v>
-      </c>
-      <c r="R11">
-        <v>65000</v>
-      </c>
-      <c r="S11" t="s">
-        <v>99</v>
-      </c>
-      <c r="T11" t="s">
-        <v>164</v>
-      </c>
-      <c r="U11">
-        <v>200000</v>
-      </c>
-      <c r="V11" t="s">
-        <v>165</v>
-      </c>
-      <c r="W11">
-        <v>53200</v>
-      </c>
-      <c r="X11" t="s">
-        <v>166</v>
-      </c>
-      <c r="Y11">
-        <v>100000</v>
-      </c>
-      <c r="AD11">
-        <v>0</v>
-      </c>
-      <c r="AE11" t="s">
-        <v>167</v>
-      </c>
-      <c r="AF11">
-        <v>24000</v>
-      </c>
-      <c r="AG11" t="s">
-        <v>55</v>
-      </c>
-      <c r="AH11">
-        <v>0</v>
-      </c>
-      <c r="AI11" t="s">
-        <v>168</v>
-      </c>
-      <c r="AJ11" t="s">
-        <v>169</v>
-      </c>
-      <c r="AK11" t="s">
-        <v>170</v>
-      </c>
-      <c r="AL11" t="s">
-        <v>77</v>
-      </c>
-      <c r="AM11" t="s">
-        <v>171</v>
-      </c>
-      <c r="AO11" t="s">
-        <v>172</v>
-      </c>
-      <c r="AP11" t="s">
-        <v>173</v>
-      </c>
-      <c r="AT11" t="s">
-        <v>174</v>
-      </c>
-      <c r="AU11" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="12" spans="1:47">
-      <c r="A12">
-        <v>44</v>
-      </c>
-      <c r="B12">
-        <v>46229.965208333299</v>
-      </c>
-      <c r="C12">
-        <v>46229.976365740702</v>
-      </c>
-      <c r="D12" t="s">
-        <v>176</v>
-      </c>
-      <c r="F12" t="s">
-        <v>47</v>
-      </c>
-      <c r="G12" t="s">
-        <v>190</v>
-      </c>
-      <c r="H12">
-        <v>46229</v>
-      </c>
-      <c r="I12" t="s">
-        <v>191</v>
+      <c r="J12">
+        <v>0</v>
       </c>
       <c r="K12">
-        <v>110000</v>
-      </c>
-      <c r="M12" t="s">
-        <v>82</v>
-      </c>
-      <c r="N12" t="s">
-        <v>71</v>
-      </c>
-      <c r="O12" t="s">
-        <v>192</v>
-      </c>
-      <c r="P12" t="s">
-        <v>73</v>
-      </c>
-      <c r="Q12" t="s">
-        <v>193</v>
-      </c>
-      <c r="R12">
-        <v>85000</v>
-      </c>
-      <c r="S12" t="s">
-        <v>54</v>
-      </c>
-      <c r="T12" t="s">
-        <v>55</v>
-      </c>
-      <c r="U12">
-        <v>0</v>
-      </c>
-      <c r="V12" t="s">
-        <v>194</v>
-      </c>
-      <c r="W12">
-        <v>0</v>
-      </c>
-      <c r="X12" t="s">
-        <v>55</v>
-      </c>
-      <c r="Y12">
-        <v>0</v>
-      </c>
-      <c r="AD12">
-        <v>0</v>
-      </c>
-      <c r="AE12" t="s">
-        <v>55</v>
-      </c>
-      <c r="AF12">
-        <v>0</v>
-      </c>
-      <c r="AG12" t="s">
-        <v>55</v>
-      </c>
-      <c r="AH12">
-        <v>0</v>
-      </c>
-      <c r="AI12" t="s">
-        <v>195</v>
-      </c>
-      <c r="AJ12" t="s">
-        <v>196</v>
-      </c>
-      <c r="AM12" t="s">
-        <v>197</v>
-      </c>
-      <c r="AN12" t="s">
-        <v>198</v>
-      </c>
-      <c r="AO12" t="s">
-        <v>199</v>
-      </c>
-      <c r="AP12" t="s">
-        <v>118</v>
-      </c>
-      <c r="AQ12" t="s">
-        <v>200</v>
-      </c>
-      <c r="AR12" t="s">
-        <v>201</v>
-      </c>
-      <c r="AS12" t="s">
-        <v>202</v>
+        <v>77000</v>
+      </c>
+      <c r="L12">
+        <v>0</v>
+      </c>
+      <c r="M12">
+        <v>80000</v>
+      </c>
+    </row>
+    <row r="13" spans="2:13">
+      <c r="B13" t="s">
+        <v>319</v>
+      </c>
+      <c r="C13">
+        <v>0</v>
+      </c>
+      <c r="D13">
+        <v>0</v>
+      </c>
+      <c r="F13">
+        <v>0</v>
+      </c>
+      <c r="G13">
+        <v>0</v>
+      </c>
+      <c r="I13">
+        <v>0</v>
+      </c>
+      <c r="K13">
+        <v>0</v>
+      </c>
+      <c r="M13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="2:13">
+      <c r="B14" t="s">
+        <v>320</v>
+      </c>
+      <c r="C14">
+        <v>0</v>
+      </c>
+      <c r="D14">
+        <v>22000</v>
+      </c>
+      <c r="F14">
+        <v>0</v>
+      </c>
+      <c r="G14">
+        <v>0</v>
+      </c>
+      <c r="H14">
+        <v>0</v>
+      </c>
+      <c r="I14">
+        <v>0</v>
+      </c>
+      <c r="J14">
+        <v>0</v>
+      </c>
+      <c r="K14">
+        <v>0</v>
+      </c>
+      <c r="L14">
+        <v>0</v>
+      </c>
+      <c r="M14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="2:13">
+      <c r="B15" t="s">
+        <v>321</v>
+      </c>
+      <c r="C15">
+        <v>22000</v>
+      </c>
+      <c r="D15">
+        <v>379000</v>
+      </c>
+      <c r="F15">
+        <v>59062.5</v>
+      </c>
+      <c r="G15">
+        <v>928750</v>
+      </c>
+      <c r="H15">
+        <v>69062.5</v>
+      </c>
+      <c r="I15">
+        <v>1088750</v>
+      </c>
+      <c r="J15">
+        <v>81062.5</v>
+      </c>
+      <c r="K15">
+        <v>1280750</v>
+      </c>
+      <c r="L15">
+        <v>84062.5</v>
+      </c>
+      <c r="M15">
+        <v>1328750</v>
       </c>
     </row>
   </sheetData>
@@ -4460,628 +3452,388 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{11CE9076-FBF7-47E4-B83B-D8B70638F4DE}">
-  <dimension ref="B2:B47"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
-  <sheetData>
-    <row r="2" spans="2:2">
-      <c r="B2" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="2:2">
-      <c r="B3" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="4" spans="2:2">
-      <c r="B4" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="5" spans="2:2">
-      <c r="B5" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="6" spans="2:2">
-      <c r="B6" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="7" spans="2:2">
-      <c r="B7" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="8" spans="2:2">
-      <c r="B8" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="9" spans="2:2">
-      <c r="B9" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="10" spans="2:2">
-      <c r="B10" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="11" spans="2:2">
-      <c r="B11" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="12" spans="2:2">
-      <c r="B12" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="13" spans="2:2">
-      <c r="B13" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="14" spans="2:2">
-      <c r="B14" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="15" spans="2:2">
-      <c r="B15" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="16" spans="2:2">
-      <c r="B16" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="17" spans="2:2">
-      <c r="B17" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="18" spans="2:2">
-      <c r="B18" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="19" spans="2:2">
-      <c r="B19" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="20" spans="2:2">
-      <c r="B20" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="21" spans="2:2">
-      <c r="B21" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="22" spans="2:2">
-      <c r="B22" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="23" spans="2:2">
-      <c r="B23" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="24" spans="2:2">
-      <c r="B24" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="25" spans="2:2">
-      <c r="B25" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="26" spans="2:2">
-      <c r="B26" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="27" spans="2:2">
-      <c r="B27" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="28" spans="2:2">
-      <c r="B28" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="29" spans="2:2">
-      <c r="B29" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="30" spans="2:2">
-      <c r="B30" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="31" spans="2:2">
-      <c r="B31" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="32" spans="2:2">
-      <c r="B32" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="33" spans="2:2">
-      <c r="B33" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="34" spans="2:2">
-      <c r="B34" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="35" spans="2:2">
-      <c r="B35" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="36" spans="2:2">
-      <c r="B36" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="37" spans="2:2">
-      <c r="B37" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="38" spans="2:2">
-      <c r="B38" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="39" spans="2:2">
-      <c r="B39" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="40" spans="2:2">
-      <c r="B40" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="41" spans="2:2">
-      <c r="B41" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="42" spans="2:2">
-      <c r="B42" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="43" spans="2:2">
-      <c r="B43" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="44" spans="2:2">
-      <c r="B44" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="45" spans="2:2">
-      <c r="B45" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="46" spans="2:2">
-      <c r="B46" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="47" spans="2:2">
-      <c r="B47" t="s">
-        <v>46</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{589C5C90-B390-4A0D-9993-2A2D1DEFC028}">
   <dimension ref="B2:C48"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="2" max="2" width="36.08984375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="69.90625" customWidth="1"/>
     <col min="3" max="3" width="33.90625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:3">
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="4" t="s">
+        <v>197</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="3" spans="2:3">
+      <c r="B3" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="4" spans="2:3">
+      <c r="B4" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="5" spans="2:3">
+      <c r="B5" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="6" spans="2:3">
+      <c r="B6" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="7" spans="2:3">
+      <c r="B7" s="5" t="s">
+        <v>202</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="8" spans="2:3">
+      <c r="B8" s="6" t="s">
+        <v>204</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="9" spans="2:3">
+      <c r="B9" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="10" spans="2:3">
+      <c r="B10" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="11" spans="2:3">
+      <c r="B11" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="12" spans="2:3">
+      <c r="B12" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="13" spans="2:3">
+      <c r="B13" s="5" t="s">
+        <v>303</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="14" spans="2:3">
+      <c r="B14" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="15" spans="2:3">
+      <c r="B15" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="16" spans="2:3">
+      <c r="B16" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="17" spans="2:3">
+      <c r="B17" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="18" spans="2:3">
+      <c r="B18" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="19" spans="2:3">
+      <c r="B19" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="20" spans="2:3">
+      <c r="B20" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="21" spans="2:3" ht="29">
+      <c r="B21" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="22" spans="2:3">
+      <c r="B22" s="5" t="s">
+        <v>218</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="23" spans="2:3">
+      <c r="B23" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="24" spans="2:3">
+      <c r="B24" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="25" spans="2:3">
+      <c r="B25" s="5" t="s">
+        <v>222</v>
+      </c>
+      <c r="C25" s="2" t="s">
         <v>223</v>
       </c>
-      <c r="C2" s="1" t="s">
+    </row>
+    <row r="26" spans="2:3" ht="29">
+      <c r="B26" s="5" t="s">
         <v>224</v>
       </c>
-    </row>
-    <row r="3" spans="2:3">
-      <c r="B3" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C3" s="3" t="s">
+      <c r="C26" s="2" t="s">
         <v>225</v>
       </c>
     </row>
-    <row r="4" spans="2:3">
-      <c r="B4" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="C4" s="3" t="s">
+    <row r="27" spans="2:3" ht="29">
+      <c r="B27" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C27" s="2" t="s">
         <v>226</v>
       </c>
     </row>
-    <row r="5" spans="2:3">
-      <c r="B5" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="C5" s="3" t="s">
+    <row r="28" spans="2:3" ht="29">
+      <c r="B28" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="C28" s="2" t="s">
         <v>227</v>
       </c>
     </row>
-    <row r="6" spans="2:3">
-      <c r="B6" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C6" s="3" t="s">
+    <row r="29" spans="2:3" ht="29">
+      <c r="B29" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="C29" s="2" t="s">
         <v>228</v>
       </c>
     </row>
-    <row r="7" spans="2:3">
-      <c r="B7" s="2" t="s">
+    <row r="30" spans="2:3" ht="29">
+      <c r="B30" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="C30" s="2" t="s">
         <v>229</v>
       </c>
-      <c r="C7" s="3" t="s">
+    </row>
+    <row r="31" spans="2:3">
+      <c r="B31" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="C31" s="2" t="s">
         <v>230</v>
       </c>
     </row>
-    <row r="8" spans="2:3">
-      <c r="B8" s="2" t="s">
+    <row r="32" spans="2:3">
+      <c r="B32" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="C32" s="2" t="s">
         <v>231</v>
       </c>
-      <c r="C8" s="3" t="s">
+    </row>
+    <row r="33" spans="2:3">
+      <c r="B33" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="C33" s="2" t="s">
         <v>232</v>
       </c>
     </row>
-    <row r="9" spans="2:3">
-      <c r="B9" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C9" s="3" t="s">
+    <row r="34" spans="2:3">
+      <c r="B34" s="5" t="s">
         <v>233</v>
       </c>
-    </row>
-    <row r="10" spans="2:3">
-      <c r="B10" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C10" s="3" t="s">
+      <c r="C34" s="2" t="s">
         <v>234</v>
       </c>
     </row>
-    <row r="11" spans="2:3">
-      <c r="B11" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C11" s="3" t="s">
+    <row r="35" spans="2:3">
+      <c r="B35" s="5" t="s">
         <v>235</v>
       </c>
-    </row>
-    <row r="12" spans="2:3">
-      <c r="B12" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="C12" s="3" t="s">
+      <c r="C35" s="2" t="s">
         <v>236</v>
       </c>
     </row>
-    <row r="13" spans="2:3">
-      <c r="B13" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C13" s="3" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="14" spans="2:3">
-      <c r="B14" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C14" s="3" t="s">
+    <row r="36" spans="2:3">
+      <c r="B36" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="C36" s="2" t="s">
         <v>237</v>
       </c>
     </row>
-    <row r="15" spans="2:3">
-      <c r="B15" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C15" s="3" t="s">
+    <row r="37" spans="2:3">
+      <c r="B37" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="C37" s="2" t="s">
         <v>238</v>
       </c>
     </row>
-    <row r="16" spans="2:3">
-      <c r="B16" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="C16" s="3" t="s">
+    <row r="38" spans="2:3">
+      <c r="B38" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="C38" s="2" t="s">
         <v>239</v>
       </c>
     </row>
-    <row r="17" spans="2:3">
-      <c r="B17" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C17" s="3" t="s">
+    <row r="39" spans="2:3">
+      <c r="B39" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="C39" s="2" t="s">
         <v>240</v>
       </c>
     </row>
-    <row r="18" spans="2:3">
-      <c r="B18" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="C18" s="3" t="s">
+    <row r="40" spans="2:3">
+      <c r="B40" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="C40" s="2" t="s">
         <v>241</v>
       </c>
     </row>
-    <row r="19" spans="2:3">
-      <c r="B19" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="C19" s="3" t="s">
+    <row r="41" spans="2:3">
+      <c r="B41" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="C41" s="2" t="s">
         <v>242</v>
       </c>
     </row>
-    <row r="20" spans="2:3">
-      <c r="B20" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="C20" s="3" t="s">
+    <row r="42" spans="2:3">
+      <c r="B42" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="C42" s="2" t="s">
         <v>243</v>
       </c>
     </row>
-    <row r="21" spans="2:3" ht="29">
-      <c r="B21" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="C21" s="3" t="s">
+    <row r="43" spans="2:3">
+      <c r="B43" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="C43" s="2" t="s">
         <v>244</v>
       </c>
     </row>
-    <row r="22" spans="2:3" ht="29">
-      <c r="B22" s="2" t="s">
+    <row r="44" spans="2:3">
+      <c r="B44" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="C44" s="2" t="s">
         <v>245</v>
       </c>
-      <c r="C22" s="3" t="s">
+    </row>
+    <row r="45" spans="2:3">
+      <c r="B45" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="C45" s="2" t="s">
         <v>246</v>
       </c>
     </row>
-    <row r="23" spans="2:3">
-      <c r="B23" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="C23" s="3" t="s">
+    <row r="46" spans="2:3">
+      <c r="B46" s="5" t="s">
         <v>247</v>
       </c>
-    </row>
-    <row r="24" spans="2:3">
-      <c r="B24" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="C24" s="3" t="s">
+      <c r="C46" s="2" t="s">
         <v>248</v>
       </c>
     </row>
-    <row r="25" spans="2:3">
-      <c r="B25" s="2" t="s">
+    <row r="47" spans="2:3">
+      <c r="B47" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="C47" s="2" t="s">
         <v>249</v>
       </c>
-      <c r="C25" s="3" t="s">
+    </row>
+    <row r="48" spans="2:3">
+      <c r="B48" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="C48" s="2" t="s">
         <v>250</v>
-      </c>
-    </row>
-    <row r="26" spans="2:3" ht="29">
-      <c r="B26" s="2" t="s">
-        <v>251</v>
-      </c>
-      <c r="C26" s="3" t="s">
-        <v>252</v>
-      </c>
-    </row>
-    <row r="27" spans="2:3" ht="29">
-      <c r="B27" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="C27" s="3" t="s">
-        <v>253</v>
-      </c>
-    </row>
-    <row r="28" spans="2:3" ht="29">
-      <c r="B28" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="C28" s="3" t="s">
-        <v>254</v>
-      </c>
-    </row>
-    <row r="29" spans="2:3" ht="29">
-      <c r="B29" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="C29" s="3" t="s">
-        <v>255</v>
-      </c>
-    </row>
-    <row r="30" spans="2:3" ht="29">
-      <c r="B30" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="C30" s="3" t="s">
-        <v>256</v>
-      </c>
-    </row>
-    <row r="31" spans="2:3">
-      <c r="B31" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="C31" s="3" t="s">
-        <v>257</v>
-      </c>
-    </row>
-    <row r="32" spans="2:3">
-      <c r="B32" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="C32" s="3" t="s">
-        <v>258</v>
-      </c>
-    </row>
-    <row r="33" spans="2:3">
-      <c r="B33" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="C33" s="3" t="s">
-        <v>259</v>
-      </c>
-    </row>
-    <row r="34" spans="2:3">
-      <c r="B34" s="2" t="s">
-        <v>260</v>
-      </c>
-      <c r="C34" s="3" t="s">
-        <v>261</v>
-      </c>
-    </row>
-    <row r="35" spans="2:3">
-      <c r="B35" s="2" t="s">
-        <v>262</v>
-      </c>
-      <c r="C35" s="3" t="s">
-        <v>263</v>
-      </c>
-    </row>
-    <row r="36" spans="2:3">
-      <c r="B36" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="C36" s="3" t="s">
-        <v>264</v>
-      </c>
-    </row>
-    <row r="37" spans="2:3">
-      <c r="B37" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="C37" s="3" t="s">
-        <v>265</v>
-      </c>
-    </row>
-    <row r="38" spans="2:3">
-      <c r="B38" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="C38" s="3" t="s">
-        <v>266</v>
-      </c>
-    </row>
-    <row r="39" spans="2:3">
-      <c r="B39" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="C39" s="3" t="s">
-        <v>267</v>
-      </c>
-    </row>
-    <row r="40" spans="2:3">
-      <c r="B40" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="C40" s="3" t="s">
-        <v>268</v>
-      </c>
-    </row>
-    <row r="41" spans="2:3">
-      <c r="B41" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="C41" s="3" t="s">
-        <v>269</v>
-      </c>
-    </row>
-    <row r="42" spans="2:3">
-      <c r="B42" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="C42" s="3" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="43" spans="2:3">
-      <c r="B43" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="C43" s="3" t="s">
-        <v>271</v>
-      </c>
-    </row>
-    <row r="44" spans="2:3">
-      <c r="B44" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="C44" s="3" t="s">
-        <v>272</v>
-      </c>
-    </row>
-    <row r="45" spans="2:3">
-      <c r="B45" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="C45" s="3" t="s">
-        <v>273</v>
-      </c>
-    </row>
-    <row r="46" spans="2:3">
-      <c r="B46" s="2" t="s">
-        <v>274</v>
-      </c>
-      <c r="C46" s="3" t="s">
-        <v>275</v>
-      </c>
-    </row>
-    <row r="47" spans="2:3">
-      <c r="B47" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="C47" s="3" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="48" spans="2:3">
-      <c r="B48" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="C48" s="3" t="s">
-        <v>277</v>
       </c>
     </row>
   </sheetData>

</xml_diff>